<commit_message>
chore: API 명세서 수정
</commit_message>
<xml_diff>
--- a/docs/TuneLog_API_명세서.xlsx
+++ b/docs/TuneLog_API_명세서.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API 명세서" sheetId="1" r:id="R42a360c5de5f482f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="수정내역" sheetId="2" r:id="R8ee52b54f14b46c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API 명세서" sheetId="1" r:id="R1a19caaac26c470b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="수정내역" sheetId="2" r:id="R1a77c30bf46a4ef8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1683,13 +1683,13 @@
     "author": "Justin",
     "author_profile_image": "/uploads/profile-justin.png",
     "image_url": "/uploads/oasis-whatever.jpg",
-    "like_count": 3,
-    "comment_count": 2,
-    "liked": true,
+    "like_count": 0,
+    "comment_count": 0,
+    "liked": false,
     "created_at": "2026-08-09T12:00:00",
     "content": "어떤 상황에서도 자유롭게 살아가자는 메시지가 좋았습니다.",
     "user_id": 1,
-    "view_count": 24,
+    "view_count": 0,
     "updated_at": "2026-08-09T12:00:00"
   }
 }</x:v>
@@ -1814,7 +1814,7 @@
     "genre": "ROCK",
     "author": "Justin",
     "author_profile_image": "/uploads/profile-justin.png",
-    "image_url": "/uploads/oasis-whatever.jpg",
+    "image_url": "/uploads/oasis-whatever-new.jpg",
     "like_count": 3,
     "comment_count": 2,
     "liked": true,
@@ -1822,7 +1822,7 @@
     "content": "수정한 감상평입니다.",
     "user_id": 1,
     "view_count": 24,
-    "updated_at": "2026-08-09T12:00:00"
+    "updated_at": "2026-08-09T12:10:00"
   }
 }</x:v>
       </x:c>

</xml_diff>